<commit_message>
Added external force model and updated powertrain model.
</commit_message>
<xml_diff>
--- a/Vehicles/F25/parameters.xlsx
+++ b/Vehicles/F25/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ryan Koo\PycharmProjects\Steady-State Lap Time Simulator\Vehicles\F25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F84FAA-329C-4E69-8653-4BB2A40BFE51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4140D785-CF83-4276-BCBE-9ECEEAEF3260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-15480" yWindow="9810" windowWidth="15600" windowHeight="11040" xr2:uid="{DAA64B5D-7408-4506-8E44-C0800644134F}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
   <si>
     <t>Parameter</t>
   </si>
@@ -54,12 +54,6 @@
     <t>Front Mass Distribution</t>
   </si>
   <si>
-    <t>Drag Coefficient Cd</t>
-  </si>
-  <si>
-    <t>Lift Coefficent Cl</t>
-  </si>
-  <si>
     <t>Front Aero Distribution</t>
   </si>
   <si>
@@ -87,9 +81,6 @@
     <t>RWD</t>
   </si>
   <si>
-    <t>FWD, RWD, or AWD</t>
-  </si>
-  <si>
     <t>Air Density is approximately this value at 20 degrees Celcius</t>
   </si>
   <si>
@@ -99,13 +90,34 @@
     <t>Tire Diameter</t>
   </si>
   <si>
-    <t>Maybe use tire's loaded diameter</t>
-  </si>
-  <si>
     <t>Tire Width</t>
   </si>
   <si>
     <t>in</t>
+  </si>
+  <si>
+    <t>Negative value always.</t>
+  </si>
+  <si>
+    <t>Positive to indicate lift. Negative to indicate downforce.</t>
+  </si>
+  <si>
+    <t>Lift Coefficent - Cl</t>
+  </si>
+  <si>
+    <t>Drag Coefficient - Cd</t>
+  </si>
+  <si>
+    <t>Rolling Resistance - Crr</t>
+  </si>
+  <si>
+    <t>Use tire's loaded diameter for better accuracy.</t>
+  </si>
+  <si>
+    <t>Enter FWD, RWD, or AWD.</t>
+  </si>
+  <si>
+    <t>Negative value always. Single tire value.</t>
   </si>
 </sst>
 </file>
@@ -471,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A669D548-F302-48C8-8201-C84AE9E0885D}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -513,7 +525,7 @@
         <v>270</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -524,12 +536,12 @@
         <v>50</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="B5" s="2">
         <v>0.1</v>
@@ -537,71 +549,77 @@
       <c r="C5" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="B6" s="2">
-        <v>0.5</v>
+        <v>-0.5</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7" s="2">
         <v>50</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="2">
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9" s="2">
         <v>1.204</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B11" s="2">
         <v>3.69</v>
@@ -612,27 +630,41 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B12" s="2">
         <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B13" s="2">
         <v>7.5</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="2">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix scalability issues and add stripping of whitespace for Excel input
</commit_message>
<xml_diff>
--- a/Vehicles/F25/parameters.xlsx
+++ b/Vehicles/F25/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ryan Koo\PycharmProjects\Steady-State Lap Time Simulator\Vehicles\F25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4140D785-CF83-4276-BCBE-9ECEEAEF3260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{927FC596-6E98-46FC-BD5F-CAED8C90BD70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-15480" yWindow="9810" windowWidth="15600" windowHeight="11040" xr2:uid="{DAA64B5D-7408-4506-8E44-C0800644134F}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="53">
   <si>
     <t>Parameter</t>
   </si>
@@ -36,9 +36,6 @@
     <t>Unit</t>
   </si>
   <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
@@ -102,15 +99,6 @@
     <t>Positive to indicate lift. Negative to indicate downforce.</t>
   </si>
   <si>
-    <t>Lift Coefficent - Cl</t>
-  </si>
-  <si>
-    <t>Drag Coefficient - Cd</t>
-  </si>
-  <si>
-    <t>Rolling Resistance - Crr</t>
-  </si>
-  <si>
     <t>Use tire's loaded diameter for better accuracy.</t>
   </si>
   <si>
@@ -118,6 +106,84 @@
   </si>
   <si>
     <t>Negative value always. Single tire value.</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Symbol</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>d_fm</t>
+  </si>
+  <si>
+    <t>d_fa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lift Coefficent </t>
+  </si>
+  <si>
+    <t>Drag Coefficient</t>
+  </si>
+  <si>
+    <t>Cl</t>
+  </si>
+  <si>
+    <t>Cd</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>rho</t>
+  </si>
+  <si>
+    <t>drive_type</t>
+  </si>
+  <si>
+    <t>Crr</t>
+  </si>
+  <si>
+    <t>Rolling Resistance</t>
+  </si>
+  <si>
+    <t>Tire Friction Coefficent Longitudinal</t>
+  </si>
+  <si>
+    <t>Tire Friction Coefficent Lateral</t>
+  </si>
+  <si>
+    <t>mu_x</t>
+  </si>
+  <si>
+    <t>mu_y</t>
+  </si>
+  <si>
+    <t>tire_d</t>
+  </si>
+  <si>
+    <t>Tire Rolling Radius</t>
+  </si>
+  <si>
+    <t>tire_roll</t>
+  </si>
+  <si>
+    <t>tire_w</t>
+  </si>
+  <si>
+    <t>idk</t>
+  </si>
+  <si>
+    <t>Friction coefficent values from optimum lap.</t>
+  </si>
+  <si>
+    <t>fdr</t>
   </si>
 </sst>
 </file>
@@ -141,12 +207,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -163,10 +235,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -483,191 +555,280 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A669D548-F302-48C8-8201-C84AE9E0885D}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.33203125" customWidth="1"/>
-    <col min="2" max="2" width="14" style="2" customWidth="1"/>
-    <col min="3" max="3" width="10.21875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="53.44140625" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="53.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="1">
+        <v>270</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2">
-        <v>270</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="1">
+        <v>50</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="1">
+        <v>-0.5</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="1">
         <v>50</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1.204</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="2">
-        <v>0.1</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="1">
+        <v>3.69</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="1">
+        <v>16</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="13" spans="1:5" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1.78</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E17" t="s">
         <v>26</v>
-      </c>
-      <c r="B6" s="2">
-        <v>-0.5</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="2">
-        <v>50</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="2">
-        <v>1</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="2">
-        <v>1.204</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="2">
-        <v>3.69</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="2">
-        <v>16</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="2">
-        <v>7.5</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="2">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement magic formula tire model and update powertrain model to compute motor tractive forces.
</commit_message>
<xml_diff>
--- a/Vehicles/F25/parameters.xlsx
+++ b/Vehicles/F25/parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ryan Koo\PycharmProjects\Steady-State Lap Time Simulator\Vehicles\F25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{927FC596-6E98-46FC-BD5F-CAED8C90BD70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FBE879D-7A51-4D57-929E-7861942F46B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15480" yWindow="9810" windowWidth="15600" windowHeight="11040" xr2:uid="{DAA64B5D-7408-4506-8E44-C0800644134F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{DAA64B5D-7408-4506-8E44-C0800644134F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="66">
   <si>
     <t>Parameter</t>
   </si>
@@ -117,9 +117,6 @@
     <t>m</t>
   </si>
   <si>
-    <t>name</t>
-  </si>
-  <si>
     <t>d_fm</t>
   </si>
   <si>
@@ -141,6 +138,12 @@
     <t>A</t>
   </si>
   <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
     <t>rho</t>
   </si>
   <si>
@@ -168,22 +171,58 @@
     <t>tire_d</t>
   </si>
   <si>
-    <t>Tire Rolling Radius</t>
-  </si>
-  <si>
-    <t>tire_roll</t>
+    <t>Tire Effective Rolling Radius</t>
   </si>
   <si>
     <t>tire_w</t>
   </si>
   <si>
-    <t>idk</t>
-  </si>
-  <si>
     <t>Friction coefficent values from optimum lap.</t>
   </si>
   <si>
     <t>fdr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name </t>
+  </si>
+  <si>
+    <t>Magic Formula - Stiffness Factor</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Magic Formula Shape Factor</t>
+  </si>
+  <si>
+    <t>Magic Formula - Peak Value</t>
+  </si>
+  <si>
+    <t>Magic Formula Curvature Factor</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>These coefficents are for the Hoosier R25 Tires</t>
+  </si>
+  <si>
+    <t>^</t>
+  </si>
+  <si>
+    <t>R_e</t>
+  </si>
+  <si>
+    <t>I just guessed this value….. Find a better one</t>
+  </si>
+  <si>
+    <t>Drivetrain Efficiency</t>
+  </si>
+  <si>
+    <t>eta</t>
+  </si>
+  <si>
+    <t>To account for drivetrain losses.</t>
   </si>
 </sst>
 </file>
@@ -233,13 +272,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -555,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A669D548-F302-48C8-8201-C84AE9E0885D}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.33203125" customWidth="1"/>
@@ -587,7 +629,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>4</v>
@@ -615,7 +657,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C4" s="1">
         <v>50</v>
@@ -626,10 +668,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="1">
         <v>0.1</v>
@@ -643,10 +685,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" s="1">
         <v>-0.5</v>
@@ -663,7 +705,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" s="1">
         <v>50</v>
@@ -677,7 +719,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" s="1">
         <v>1</v>
@@ -691,7 +733,7 @@
         <v>10</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C9" s="1">
         <v>1.204</v>
@@ -708,7 +750,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>16</v>
@@ -725,7 +767,7 @@
         <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C11" s="1">
         <v>3.69</v>
@@ -736,64 +778,67 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="1">
+        <v>0.9</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="1">
+      <c r="B13" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="1">
         <v>16</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="1">
-        <v>7.5</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="14" spans="1:5" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="C14" s="1">
+        <v>7.5</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C15" s="1">
-        <v>1.7</v>
+        <v>7</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E15" t="s">
-        <v>51</v>
+        <v>21</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -804,27 +849,112 @@
         <v>45</v>
       </c>
       <c r="C16" s="1">
-        <v>1.78</v>
+        <v>1.7</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1.78</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C17" s="1">
+      <c r="C18" s="1">
         <v>0.02</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="D18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E18" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0.1404</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1.3268</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" s="1">
+        <v>2763.46</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="1">
+        <v>-1.6122000000000001</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>